<commit_message>
Deploying to gh-pages from @ pimborman/nixie-clock@f2f99fc9c055b6a24ea9afff4494f699b42b19b0 🚀
</commit_message>
<xml_diff>
--- a/BoM/Positional/nixie-bom.xlsx
+++ b/BoM/Positional/nixie-bom.xlsx
@@ -152,7 +152,7 @@
     <t>2.0000</t>
   </si>
   <si>
-    <t>GND,Net-(BT1-+)</t>
+    <t>Net-(BT1-+),GND</t>
   </si>
   <si>
     <t>Default</t>
@@ -227,7 +227,7 @@
     <t>6.6000</t>
   </si>
   <si>
-    <t>ROT_A,GND</t>
+    <t>GND,ROT_A</t>
   </si>
   <si>
     <t>4</t>
@@ -254,7 +254,7 @@
     <t>270.0000</t>
   </si>
   <si>
-    <t>Vin,GND</t>
+    <t>GND,Vin</t>
   </si>
   <si>
     <t>5</t>
@@ -287,7 +287,7 @@
     <t>HV,GND</t>
   </si>
   <si>
-    <t>Default,HV</t>
+    <t>HV,Default</t>
   </si>
   <si>
     <t>6</t>
@@ -341,7 +341,7 @@
     <t>9.2200</t>
   </si>
   <si>
-    <t>Net-(D1-K),Net-(D1-A)</t>
+    <t>Net-(D1-A),Net-(D1-K)</t>
   </si>
   <si>
     <t>8</t>
@@ -377,7 +377,7 @@
     <t>2.4000</t>
   </si>
   <si>
-    <t>Net-(D3-A2),GND</t>
+    <t>GND,Net-(D3-A2)</t>
   </si>
   <si>
     <t>D</t>
@@ -401,7 +401,7 @@
     <t>2.2000</t>
   </si>
   <si>
-    <t>Net-(D2-A),HV</t>
+    <t>HV,Net-(D2-A)</t>
   </si>
   <si>
     <t>10</t>
@@ -527,7 +527,7 @@
     <t>13.5433</t>
   </si>
   <si>
-    <t>Net-(N1-PadA),/D15,unconnected-(N1-PadRHDP),/D13,/D12,/D16,/D14,/D17,/D19,/D110,unconnected-(N1-PadLHDP),/D11,/D18</t>
+    <t>unconnected-(N1-PadRHDP),/D15,Net-(N1-PadA),unconnected-(N1-PadLHDP),/D16,/D13,/D11,/D18,/D110,/D17,/D12,/D19,/D14</t>
   </si>
   <si>
     <t>14</t>
@@ -596,7 +596,7 @@
     <t>1.5000</t>
   </si>
   <si>
-    <t>GND,Net-(D1-K),Net-(D1-A)</t>
+    <t>Net-(D1-A),GND,Net-(D1-K)</t>
   </si>
   <si>
     <t>16</t>
@@ -632,7 +632,7 @@
     <t>19.4100</t>
   </si>
   <si>
-    <t>,Net-(D2-A),Net-(D1-K),GND</t>
+    <t>,GND,Net-(D1-K),Net-(D2-A)</t>
   </si>
   <si>
     <t>17</t>
@@ -656,7 +656,7 @@
     <t>-90.0000</t>
   </si>
   <si>
-    <t>GND,Net-(D1-A)</t>
+    <t>Net-(D1-A),GND</t>
   </si>
   <si>
     <t>18</t>
@@ -692,7 +692,7 @@
     <t>-75.6000</t>
   </si>
   <si>
-    <t>Net-(R16-Pad2),ROT_A</t>
+    <t>ROT_A,Net-(R16-Pad2)</t>
   </si>
   <si>
     <t>20</t>
@@ -713,7 +713,7 @@
     <t>-105.8100</t>
   </si>
   <si>
-    <t>Net-(N1-PadA),HV</t>
+    <t>HV,Net-(N1-PadA)</t>
   </si>
   <si>
     <t>21</t>
@@ -776,7 +776,7 @@
     <t>16.0000</t>
   </si>
   <si>
-    <t>,Net-(R18-Pad2),Net-(R21-Pad2),Net-(R16-Pad2),GND</t>
+    <t>,Net-(R16-Pad2),Net-(R21-Pad2),GND,Net-(R18-Pad2)</t>
   </si>
   <si>
     <t>23</t>
@@ -812,7 +812,7 @@
     <t>19.3800</t>
   </si>
   <si>
-    <t>Net-(U1-Aout),5V,Net-(U1-Cout),Net-(U1-Bout),DATA_IN,GND,OE,unconnected-(U1-Dout-Pad10),unconnected-(U1-Fout-Pad15),unconnected-(U1-Eout-Pad12),Vin,CLK</t>
+    <t>CLK,Net-(U1-Aout),unconnected-(U1-Eout-Pad12),Net-(U1-Cout),Vin,unconnected-(U1-Fout-Pad15),unconnected-(U1-Dout-Pad10),OE,Net-(U1-Bout),DATA_IN,GND,5V</t>
   </si>
   <si>
     <t>24</t>
@@ -845,7 +845,7 @@
     <t>34.6200</t>
   </si>
   <si>
-    <t>unconnected-(U6-PD0-Pad2),SQW,unconnected-(U6-PC3-Pad26),DATA_IN,SDA,CLK,unconnected-(U6-PC5-Pad28),unconnected-(U6-~{RESET}{slash}PC6-Pad1),ROT_PSH,GND,unconnected-(U6-XTAL2{slash}PB7-Pad10),SCL,unconnected-(U6-PC0-Pad23),unconnected-(U6-PD3-Pad5),unconnected-(U6-XTAL1{slash}PB6-Pad9),unconnected-(U6-PC1-Pad24),OE,ROT_A,unconnected-(U6-PD1-Pad3),unconnected-(U6-PC4-Pad27),unconnected-(U6-PC2-Pad25),unconnected-(U6-AREF-Pad21),ROT_B,5V,unconnected-(U6-PB5-Pad19),unconnected-(U6-PD4-Pad6)</t>
+    <t>unconnected-(U6-PC5-Pad28),unconnected-(U6-PB5-Pad19),unconnected-(U6-PD0-Pad2),unconnected-(U6-~{RESET}{slash}PC6-Pad1),unconnected-(U6-PD4-Pad6),unconnected-(U6-PC2-Pad25),SDA,unconnected-(U6-PC3-Pad26),ROT_A,unconnected-(U6-XTAL2{slash}PB7-Pad10),unconnected-(U6-PC1-Pad24),DATA_IN,ROT_B,unconnected-(U6-XTAL1{slash}PB6-Pad9),unconnected-(U6-PC0-Pad23),GND,CLK,ROT_PSH,OE,SQW,unconnected-(U6-PD3-Pad5),unconnected-(U6-PD1-Pad3),SCL,unconnected-(U6-PC4-Pad27),unconnected-(U6-AREF-Pad21),5V</t>
   </si>
   <si>
     <t>25</t>
@@ -887,7 +887,7 @@
     <t>4.4100</t>
   </si>
   <si>
-    <t>SQW,5V,GND,Net-(BT1-+),unconnected-(U7-~{RST}-Pad4),SCL,SDA,unconnected-(U7-32KHZ-Pad1)</t>
+    <t>SDA,unconnected-(U7-32KHZ-Pad1),unconnected-(U7-~{RST}-Pad4),SCL,Net-(BT1-+),GND,SQW,5V</t>
   </si>
   <si>
     <t>26</t>
@@ -923,7 +923,7 @@
     <t>13.6000</t>
   </si>
   <si>
-    <t>unconnected-(U3-NC_5-Pad34),/D120,/D116,/D121,/D16,/D131,/D117,/D14,/D119,/D114,/D111,unconnected-(U3-NC_2-Pad25),/D129,unconnected-(U3-NC_3-Pad26),Net-(U3-DATA_OUT),/D13,/D130,Net-(U1-Cout),GND,/D19,/D17,/D128,Vin,/D110,/D123,/D126,/D15,/D112,/D118,/D115,/D122,/D113,/D132,/D11,Net-(U1-Aout),/D127,unconnected-(U3-NC_1-Pad24),/D12,/D125,/D124,Net-(U1-Bout),unconnected-(U3-NC_4-Pad27),/D18</t>
+    <t>/D121,/D131,Vin,Net-(U1-Cout),unconnected-(U3-NC_2-Pad25),unconnected-(U3-NC_3-Pad26),/D118,/D117,/D127,/D114,/D126,unconnected-(U3-NC_4-Pad27),/D124,/D119,/D125,/D129,/D110,/D17,GND,/D113,/D16,/D13,unconnected-(U3-NC_1-Pad24),/D120,/D116,Net-(U1-Bout),Net-(U3-DATA_OUT),/D12,/D128,/D111,/D15,Net-(U1-Aout),/D130,unconnected-(U3-NC_5-Pad34),/D11,/D112,/D122,/D18,/D132,/D123,/D115,/D19,/D14</t>
   </si>
   <si>
     <t>27</t>
@@ -950,7 +950,7 @@
     <t>-76.9400</t>
   </si>
   <si>
-    <t>,5V,Vin,GND</t>
+    <t>,GND,5V,Vin</t>
   </si>
   <si>
     <t>28</t>
@@ -980,7 +980,7 @@
     <t>-75.0000</t>
   </si>
   <si>
-    <t>Net-(U2-TC),GND,Net-(D1-A),Vin,Net-(U2-Vfb)</t>
+    <t>Net-(U2-TC),Net-(U2-Vfb),Vin,Net-(D1-A),GND</t>
   </si>
   <si>
     <t>KiBot Bill of Materials</t>
@@ -2668,7 +2668,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:25" ht="45" customHeight="1">
+    <row r="21" spans="1:25" ht="30" customHeight="1">
       <c r="A21" s="5" t="s">
         <v>159</v>
       </c>
@@ -3669,7 +3669,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="34" spans="1:25" ht="135" customHeight="1">
+    <row r="34" spans="1:25" ht="120" customHeight="1">
       <c r="A34" s="9" t="s">
         <v>290</v>
       </c>

</xml_diff>